<commit_message>
Update KBO data 2015-2026 months 01-12
</commit_message>
<xml_diff>
--- a/data/output/kbo_postseason_schedule.xlsx
+++ b/data/output/kbo_postseason_schedule.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ162"/>
+  <dimension ref="A1:BZ164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,20 +849,16 @@
       <c r="J2" t="n">
         <v>26</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K2" t="n">
+        <v>10</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>2015-10-07</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>20151007</t>
-        </is>
+      <c r="M2" t="n">
+        <v>20151007</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -1113,20 +1109,16 @@
       <c r="J3" t="n">
         <v>7</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K3" t="n">
+        <v>10</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>2015-10-10</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>20151010</t>
-        </is>
+      <c r="M3" t="n">
+        <v>20151010</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -1373,20 +1365,16 @@
       <c r="J4" t="n">
         <v>8</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K4" t="n">
+        <v>10</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>2015-10-11</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>20151011</t>
-        </is>
+      <c r="M4" t="n">
+        <v>20151011</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -1627,20 +1615,16 @@
       <c r="J5" t="n">
         <v>9</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K5" t="n">
+        <v>10</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>2015-10-13</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>20151013</t>
-        </is>
+      <c r="M5" t="n">
+        <v>20151013</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1881,20 +1865,16 @@
       <c r="J6" t="n">
         <v>10</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K6" t="n">
+        <v>10</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>2015-10-14</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>20151014</t>
-        </is>
+      <c r="M6" t="n">
+        <v>20151014</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -2137,20 +2117,16 @@
       <c r="J7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K7" t="n">
+        <v>10</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>2015-10-18</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>20151018</t>
-        </is>
+      <c r="M7" t="n">
+        <v>20151018</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -2393,20 +2369,16 @@
       <c r="J8" t="n">
         <v>13</v>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K8" t="n">
+        <v>10</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>2015-10-19</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>20151019</t>
-        </is>
+      <c r="M8" t="n">
+        <v>20151019</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -2647,20 +2619,16 @@
       <c r="J9" t="n">
         <v>14</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K9" t="n">
+        <v>10</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>2015-10-21</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>20151021</t>
-        </is>
+      <c r="M9" t="n">
+        <v>20151021</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -2903,20 +2871,16 @@
       <c r="J10" t="n">
         <v>15</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K10" t="n">
+        <v>10</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>2015-10-22</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>20151022</t>
-        </is>
+      <c r="M10" t="n">
+        <v>20151022</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -3157,20 +3121,16 @@
       <c r="J11" t="n">
         <v>16</v>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K11" t="n">
+        <v>10</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>2015-10-24</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>20151024</t>
-        </is>
+      <c r="M11" t="n">
+        <v>20151024</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -3413,20 +3373,16 @@
       <c r="J12" t="n">
         <v>19</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K12" t="n">
+        <v>10</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>2015-10-26</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>20151026</t>
-        </is>
+      <c r="M12" t="n">
+        <v>20151026</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -3667,20 +3623,16 @@
       <c r="J13" t="n">
         <v>20</v>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K13" t="n">
+        <v>10</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>2015-10-27</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>20151027</t>
-        </is>
+      <c r="M13" t="n">
+        <v>20151027</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3923,20 +3875,16 @@
       <c r="J14" t="n">
         <v>21</v>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K14" t="n">
+        <v>10</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>2015-10-29</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>20151029</t>
-        </is>
+      <c r="M14" t="n">
+        <v>20151029</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -4177,20 +4125,16 @@
       <c r="J15" t="n">
         <v>22</v>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K15" t="n">
+        <v>10</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>2015-10-30</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>20151030</t>
-        </is>
+      <c r="M15" t="n">
+        <v>20151030</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -4431,20 +4375,16 @@
       <c r="J16" t="n">
         <v>23</v>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K16" t="n">
+        <v>10</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>2015-10-31</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>20151031</t>
-        </is>
+      <c r="M16" t="n">
+        <v>20151031</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -4685,20 +4625,16 @@
       <c r="J17" t="n">
         <v>26</v>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K17" t="n">
+        <v>10</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>2016-10-10</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>20161010</t>
-        </is>
+      <c r="M17" t="n">
+        <v>20161010</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -4941,20 +4877,16 @@
       <c r="J18" t="n">
         <v>27</v>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K18" t="n">
+        <v>10</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>2016-10-11</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>20161011</t>
-        </is>
+      <c r="M18" t="n">
+        <v>20161011</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -5197,20 +5129,16 @@
       <c r="J19" t="n">
         <v>7</v>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K19" t="n">
+        <v>10</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>2016-10-13</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>20161013</t>
-        </is>
+      <c r="M19" t="n">
+        <v>20161013</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -5453,20 +5381,16 @@
       <c r="J20" t="n">
         <v>8</v>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K20" t="n">
+        <v>10</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>2016-10-14</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>20161014</t>
-        </is>
+      <c r="M20" t="n">
+        <v>20161014</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -5707,20 +5631,16 @@
       <c r="J21" t="n">
         <v>9</v>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K21" t="n">
+        <v>10</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>2016-10-16</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>20161016</t>
-        </is>
+      <c r="M21" t="n">
+        <v>20161016</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -5961,20 +5881,16 @@
       <c r="J22" t="n">
         <v>10</v>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K22" t="n">
+        <v>10</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>2016-10-17</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>20161017</t>
-        </is>
+      <c r="M22" t="n">
+        <v>20161017</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -6215,20 +6131,16 @@
       <c r="J23" t="n">
         <v>12</v>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K23" t="n">
+        <v>10</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>2016-10-21</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>20161021</t>
-        </is>
+      <c r="M23" t="n">
+        <v>20161021</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -6471,20 +6383,16 @@
       <c r="J24" t="n">
         <v>13</v>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K24" t="n">
+        <v>10</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>2016-10-22</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>20161022</t>
-        </is>
+      <c r="M24" t="n">
+        <v>20161022</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -6725,20 +6633,16 @@
       <c r="J25" t="n">
         <v>14</v>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K25" t="n">
+        <v>10</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>2016-10-24</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>20161024</t>
-        </is>
+      <c r="M25" t="n">
+        <v>20161024</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -6989,20 +6893,16 @@
       <c r="J26" t="n">
         <v>15</v>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K26" t="n">
+        <v>10</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>2016-10-25</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>20161025</t>
-        </is>
+      <c r="M26" t="n">
+        <v>20161025</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -7245,20 +7145,16 @@
       <c r="J27" t="n">
         <v>19</v>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K27" t="n">
+        <v>10</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>2016-10-29</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>20161029</t>
-        </is>
+      <c r="M27" t="n">
+        <v>20161029</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -7509,20 +7405,16 @@
       <c r="J28" t="n">
         <v>20</v>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K28" t="n">
+        <v>10</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>2016-10-30</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>20161030</t>
-        </is>
+      <c r="M28" t="n">
+        <v>20161030</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -7763,20 +7655,16 @@
       <c r="J29" t="n">
         <v>21</v>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K29" t="n">
+        <v>11</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>2016-11-01</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>20161101</t>
-        </is>
+      <c r="M29" t="n">
+        <v>20161101</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -8019,20 +7907,16 @@
       <c r="J30" t="n">
         <v>22</v>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K30" t="n">
+        <v>11</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>2016-11-02</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>20161102</t>
-        </is>
+      <c r="M30" t="n">
+        <v>20161102</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -8275,20 +8159,16 @@
       <c r="J31" t="n">
         <v>26</v>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K31" t="n">
+        <v>10</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>2017-10-05</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>20171005</t>
-        </is>
+      <c r="M31" t="n">
+        <v>20171005</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -8529,20 +8409,16 @@
       <c r="J32" t="n">
         <v>7</v>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K32" t="n">
+        <v>10</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>2017-10-08</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>20171008</t>
-        </is>
+      <c r="M32" t="n">
+        <v>20171008</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -8793,20 +8669,16 @@
       <c r="J33" t="n">
         <v>8</v>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K33" t="n">
+        <v>10</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>2017-10-09</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>20171009</t>
-        </is>
+      <c r="M33" t="n">
+        <v>20171009</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -9047,20 +8919,16 @@
       <c r="J34" t="n">
         <v>9</v>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K34" t="n">
+        <v>10</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>2017-10-11</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>20171011</t>
-        </is>
+      <c r="M34" t="n">
+        <v>20171011</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -9301,20 +9169,16 @@
       <c r="J35" t="n">
         <v>10</v>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K35" t="n">
+        <v>10</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>2017-10-12</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>20171012</t>
-        </is>
+      <c r="M35" t="n">
+        <v>20171012</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -9463,20 +9327,16 @@
       <c r="J36" t="n">
         <v>10</v>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K36" t="n">
+        <v>10</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>2017-10-13</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>20171013</t>
-        </is>
+      <c r="M36" t="n">
+        <v>20171013</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -9719,20 +9579,16 @@
       <c r="J37" t="n">
         <v>11</v>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K37" t="n">
+        <v>10</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>2017-10-15</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>20171015</t>
-        </is>
+      <c r="M37" t="n">
+        <v>20171015</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -9975,20 +9831,16 @@
       <c r="J38" t="n">
         <v>12</v>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K38" t="n">
+        <v>10</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>2017-10-17</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>20171017</t>
-        </is>
+      <c r="M38" t="n">
+        <v>20171017</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -10231,20 +10083,16 @@
       <c r="J39" t="n">
         <v>13</v>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K39" t="n">
+        <v>10</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>2017-10-18</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>20171018</t>
-        </is>
+      <c r="M39" t="n">
+        <v>20171018</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -10485,20 +10333,16 @@
       <c r="J40" t="n">
         <v>14</v>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K40" t="n">
+        <v>10</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>2017-10-20</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>20171020</t>
-        </is>
+      <c r="M40" t="n">
+        <v>20171020</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -10741,20 +10585,16 @@
       <c r="J41" t="n">
         <v>15</v>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K41" t="n">
+        <v>10</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>2017-10-21</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>20171021</t>
-        </is>
+      <c r="M41" t="n">
+        <v>20171021</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -10997,20 +10837,16 @@
       <c r="J42" t="n">
         <v>19</v>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K42" t="n">
+        <v>10</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>2017-10-25</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>20171025</t>
-        </is>
+      <c r="M42" t="n">
+        <v>20171025</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -11253,20 +11089,16 @@
       <c r="J43" t="n">
         <v>20</v>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K43" t="n">
+        <v>10</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>2017-10-26</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>20171026</t>
-        </is>
+      <c r="M43" t="n">
+        <v>20171026</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -11507,20 +11339,16 @@
       <c r="J44" t="n">
         <v>21</v>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K44" t="n">
+        <v>10</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>2017-10-28</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>20171028</t>
-        </is>
+      <c r="M44" t="n">
+        <v>20171028</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -11763,20 +11591,16 @@
       <c r="J45" t="n">
         <v>22</v>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K45" t="n">
+        <v>10</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>2017-10-29</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>20171029</t>
-        </is>
+      <c r="M45" t="n">
+        <v>20171029</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -12019,20 +11843,16 @@
       <c r="J46" t="n">
         <v>23</v>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K46" t="n">
+        <v>10</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>2017-10-30</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>20171030</t>
-        </is>
+      <c r="M46" t="n">
+        <v>20171030</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -12275,20 +12095,16 @@
       <c r="J47" t="n">
         <v>26</v>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K47" t="n">
+        <v>10</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>2018-10-16</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>20181016</t>
-        </is>
+      <c r="M47" t="n">
+        <v>20181016</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -12529,20 +12345,16 @@
       <c r="J48" t="n">
         <v>7</v>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K48" t="n">
+        <v>10</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>2018-10-19</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>20181019</t>
-        </is>
+      <c r="M48" t="n">
+        <v>20181019</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -12785,20 +12597,16 @@
       <c r="J49" t="n">
         <v>8</v>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K49" t="n">
+        <v>10</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>2018-10-20</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>20181020</t>
-        </is>
+      <c r="M49" t="n">
+        <v>20181020</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -13041,20 +12849,16 @@
       <c r="J50" t="n">
         <v>9</v>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K50" t="n">
+        <v>10</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>2018-10-22</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>20181022</t>
-        </is>
+      <c r="M50" t="n">
+        <v>20181022</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -13297,20 +13101,16 @@
       <c r="J51" t="n">
         <v>10</v>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K51" t="n">
+        <v>10</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>2018-10-23</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>20181023</t>
-        </is>
+      <c r="M51" t="n">
+        <v>20181023</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -13551,20 +13351,16 @@
       <c r="J52" t="n">
         <v>12</v>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K52" t="n">
+        <v>10</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>2018-10-27</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>20181027</t>
-        </is>
+      <c r="M52" t="n">
+        <v>20181027</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -13807,20 +13603,16 @@
       <c r="J53" t="n">
         <v>13</v>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K53" t="n">
+        <v>10</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>2018-10-28</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>20181028</t>
-        </is>
+      <c r="M53" t="n">
+        <v>20181028</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -14061,20 +13853,16 @@
       <c r="J54" t="n">
         <v>14</v>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K54" t="n">
+        <v>10</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>2018-10-30</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>20181030</t>
-        </is>
+      <c r="M54" t="n">
+        <v>20181030</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -14315,20 +14103,16 @@
       <c r="J55" t="n">
         <v>15</v>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K55" t="n">
+        <v>10</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>2018-10-31</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>20181031</t>
-        </is>
+      <c r="M55" t="n">
+        <v>20181031</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -14569,20 +14353,16 @@
       <c r="J56" t="n">
         <v>16</v>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K56" t="n">
+        <v>11</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>2018-11-02</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>20181102</t>
-        </is>
+      <c r="M56" t="n">
+        <v>20181102</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -14829,20 +14609,16 @@
       <c r="J57" t="n">
         <v>19</v>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K57" t="n">
+        <v>11</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>2018-11-04</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>20181104</t>
-        </is>
+      <c r="M57" t="n">
+        <v>20181104</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -15085,20 +14861,16 @@
       <c r="J58" t="n">
         <v>20</v>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K58" t="n">
+        <v>11</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>2018-11-05</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>20181105</t>
-        </is>
+      <c r="M58" t="n">
+        <v>20181105</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -15339,20 +15111,16 @@
       <c r="J59" t="n">
         <v>21</v>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K59" t="n">
+        <v>11</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>2018-11-07</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>20181107</t>
-        </is>
+      <c r="M59" t="n">
+        <v>20181107</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -15593,20 +15361,16 @@
       <c r="J60" t="n">
         <v>22</v>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K60" t="n">
+        <v>11</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>2018-11-08</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>20181108</t>
-        </is>
+      <c r="M60" t="n">
+        <v>20181108</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -15755,20 +15519,16 @@
       <c r="J61" t="n">
         <v>22</v>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K61" t="n">
+        <v>11</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>2018-11-09</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>20181109</t>
-        </is>
+      <c r="M61" t="n">
+        <v>20181109</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -16011,20 +15771,16 @@
       <c r="J62" t="n">
         <v>23</v>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K62" t="n">
+        <v>11</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>2018-11-10</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>20181110</t>
-        </is>
+      <c r="M62" t="n">
+        <v>20181110</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -16265,20 +16021,16 @@
       <c r="J63" t="n">
         <v>24</v>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K63" t="n">
+        <v>11</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>2018-11-12</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>20181112</t>
-        </is>
+      <c r="M63" t="n">
+        <v>20181112</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -16533,20 +16285,16 @@
       <c r="J64" t="n">
         <v>26</v>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K64" t="n">
+        <v>10</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>2019-10-03</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>20191003</t>
-        </is>
+      <c r="M64" t="n">
+        <v>20191003</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
@@ -16787,20 +16535,16 @@
       <c r="J65" t="n">
         <v>7</v>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K65" t="n">
+        <v>10</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>2019-10-06</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>20191006</t>
-        </is>
+      <c r="M65" t="n">
+        <v>20191006</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -17043,20 +16787,16 @@
       <c r="J66" t="n">
         <v>8</v>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K66" t="n">
+        <v>10</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>2019-10-07</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>20191007</t>
-        </is>
+      <c r="M66" t="n">
+        <v>20191007</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -17303,20 +17043,16 @@
       <c r="J67" t="n">
         <v>9</v>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K67" t="n">
+        <v>10</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
           <t>2019-10-09</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>20191009</t>
-        </is>
+      <c r="M67" t="n">
+        <v>20191009</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -17557,20 +17293,16 @@
       <c r="J68" t="n">
         <v>10</v>
       </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K68" t="n">
+        <v>10</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>2019-10-10</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>20191010</t>
-        </is>
+      <c r="M68" t="n">
+        <v>20191010</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -17813,20 +17545,16 @@
       <c r="J69" t="n">
         <v>12</v>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K69" t="n">
+        <v>10</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>2019-10-14</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>20191014</t>
-        </is>
+      <c r="M69" t="n">
+        <v>20191014</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -18077,20 +17805,16 @@
       <c r="J70" t="n">
         <v>13</v>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K70" t="n">
+        <v>10</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>2019-10-15</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>20191015</t>
-        </is>
+      <c r="M70" t="n">
+        <v>20191015</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -18333,20 +18057,16 @@
       <c r="J71" t="n">
         <v>14</v>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K71" t="n">
+        <v>10</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>2019-10-17</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>20191017</t>
-        </is>
+      <c r="M71" t="n">
+        <v>20191017</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -18587,20 +18307,16 @@
       <c r="J72" t="n">
         <v>19</v>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K72" t="n">
+        <v>10</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>2019-10-22</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>20191022</t>
-        </is>
+      <c r="M72" t="n">
+        <v>20191022</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -18843,20 +18559,16 @@
       <c r="J73" t="n">
         <v>20</v>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K73" t="n">
+        <v>10</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
           <t>2019-10-23</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>20191023</t>
-        </is>
+      <c r="M73" t="n">
+        <v>20191023</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
@@ -19099,20 +18811,16 @@
       <c r="J74" t="n">
         <v>21</v>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K74" t="n">
+        <v>10</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
           <t>2019-10-25</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>20191025</t>
-        </is>
+      <c r="M74" t="n">
+        <v>20191025</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -19355,20 +19063,16 @@
       <c r="J75" t="n">
         <v>22</v>
       </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K75" t="n">
+        <v>10</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
           <t>2019-10-26</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>20191026</t>
-        </is>
+      <c r="M75" t="n">
+        <v>20191026</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -19615,20 +19319,16 @@
       <c r="J76" t="n">
         <v>26</v>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K76" t="n">
+        <v>11</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>2020-11-01</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t>20201101</t>
-        </is>
+      <c r="M76" t="n">
+        <v>20201101</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -19777,20 +19477,16 @@
       <c r="J77" t="n">
         <v>26</v>
       </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K77" t="n">
+        <v>11</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>2020-11-02</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>20201102</t>
-        </is>
+      <c r="M77" t="n">
+        <v>20201102</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -20045,20 +19741,16 @@
       <c r="J78" t="n">
         <v>7</v>
       </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K78" t="n">
+        <v>11</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>2020-11-04</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>20201104</t>
-        </is>
+      <c r="M78" t="n">
+        <v>20201104</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -20299,20 +19991,16 @@
       <c r="J79" t="n">
         <v>8</v>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K79" t="n">
+        <v>11</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>2020-11-05</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>20201105</t>
-        </is>
+      <c r="M79" t="n">
+        <v>20201105</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -20555,20 +20243,16 @@
       <c r="J80" t="n">
         <v>12</v>
       </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K80" t="n">
+        <v>11</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
           <t>2020-11-09</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>20201109</t>
-        </is>
+      <c r="M80" t="n">
+        <v>20201109</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -20811,20 +20495,16 @@
       <c r="J81" t="n">
         <v>13</v>
       </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K81" t="n">
+        <v>11</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
           <t>2020-11-10</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>20201110</t>
-        </is>
+      <c r="M81" t="n">
+        <v>20201110</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -21067,20 +20747,16 @@
       <c r="J82" t="n">
         <v>14</v>
       </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K82" t="n">
+        <v>11</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
           <t>2020-11-12</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>20201112</t>
-        </is>
+      <c r="M82" t="n">
+        <v>20201112</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -21323,20 +20999,16 @@
       <c r="J83" t="n">
         <v>15</v>
       </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K83" t="n">
+        <v>11</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
           <t>2020-11-13</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>20201113</t>
-        </is>
+      <c r="M83" t="n">
+        <v>20201113</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -21577,20 +21249,16 @@
       <c r="J84" t="n">
         <v>19</v>
       </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K84" t="n">
+        <v>11</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
           <t>2020-11-17</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>20201117</t>
-        </is>
+      <c r="M84" t="n">
+        <v>20201117</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -21831,20 +21499,16 @@
       <c r="J85" t="n">
         <v>20</v>
       </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K85" t="n">
+        <v>11</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
           <t>2020-11-18</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>20201118</t>
-        </is>
+      <c r="M85" t="n">
+        <v>20201118</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -22087,20 +21751,16 @@
       <c r="J86" t="n">
         <v>21</v>
       </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K86" t="n">
+        <v>11</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
           <t>2020-11-20</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>20201120</t>
-        </is>
+      <c r="M86" t="n">
+        <v>20201120</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -22341,20 +22001,16 @@
       <c r="J87" t="n">
         <v>22</v>
       </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K87" t="n">
+        <v>11</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
           <t>2020-11-21</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>20201121</t>
-        </is>
+      <c r="M87" t="n">
+        <v>20201121</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -22597,20 +22253,16 @@
       <c r="J88" t="n">
         <v>23</v>
       </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K88" t="n">
+        <v>11</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
           <t>2020-11-23</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>20201123</t>
-        </is>
+      <c r="M88" t="n">
+        <v>20201123</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -22851,20 +22503,16 @@
       <c r="J89" t="n">
         <v>24</v>
       </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K89" t="n">
+        <v>11</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
           <t>2020-11-24</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
-        <is>
-          <t>20201124</t>
-        </is>
+      <c r="M89" t="n">
+        <v>20201124</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -23105,20 +22753,16 @@
       <c r="J90" t="n">
         <v>26</v>
       </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K90" t="n">
+        <v>11</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
           <t>2021-11-01</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr">
-        <is>
-          <t>20211101</t>
-        </is>
+      <c r="M90" t="n">
+        <v>20211101</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -23361,20 +23005,16 @@
       <c r="J91" t="n">
         <v>27</v>
       </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K91" t="n">
+        <v>11</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
           <t>2021-11-02</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t>20211102</t>
-        </is>
+      <c r="M91" t="n">
+        <v>20211102</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -23615,20 +23255,16 @@
       <c r="J92" t="n">
         <v>7</v>
       </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K92" t="n">
+        <v>11</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
           <t>2021-11-04</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr">
-        <is>
-          <t>20211104</t>
-        </is>
+      <c r="M92" t="n">
+        <v>20211104</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -23871,20 +23507,16 @@
       <c r="J93" t="n">
         <v>8</v>
       </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K93" t="n">
+        <v>11</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
           <t>2021-11-05</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>20211105</t>
-        </is>
+      <c r="M93" t="n">
+        <v>20211105</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -24127,20 +23759,16 @@
       <c r="J94" t="n">
         <v>9</v>
       </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K94" t="n">
+        <v>11</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
           <t>2021-11-07</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr">
-        <is>
-          <t>20211107</t>
-        </is>
+      <c r="M94" t="n">
+        <v>20211107</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -24383,20 +24011,16 @@
       <c r="J95" t="n">
         <v>12</v>
       </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K95" t="n">
+        <v>11</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
           <t>2021-11-09</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>20211109</t>
-        </is>
+      <c r="M95" t="n">
+        <v>20211109</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -24639,20 +24263,16 @@
       <c r="J96" t="n">
         <v>13</v>
       </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K96" t="n">
+        <v>11</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
           <t>2021-11-10</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr">
-        <is>
-          <t>20211110</t>
-        </is>
+      <c r="M96" t="n">
+        <v>20211110</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -24893,20 +24513,16 @@
       <c r="J97" t="n">
         <v>19</v>
       </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K97" t="n">
+        <v>11</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
           <t>2021-11-14</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr">
-        <is>
-          <t>20211114</t>
-        </is>
+      <c r="M97" t="n">
+        <v>20211114</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -25147,20 +24763,16 @@
       <c r="J98" t="n">
         <v>20</v>
       </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K98" t="n">
+        <v>11</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
           <t>2021-11-15</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr">
-        <is>
-          <t>20211115</t>
-        </is>
+      <c r="M98" t="n">
+        <v>20211115</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -25401,20 +25013,16 @@
       <c r="J99" t="n">
         <v>21</v>
       </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K99" t="n">
+        <v>11</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
           <t>2021-11-17</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr">
-        <is>
-          <t>20211117</t>
-        </is>
+      <c r="M99" t="n">
+        <v>20211117</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -25657,20 +25265,16 @@
       <c r="J100" t="n">
         <v>22</v>
       </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K100" t="n">
+        <v>11</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
           <t>2021-11-18</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr">
-        <is>
-          <t>20211118</t>
-        </is>
+      <c r="M100" t="n">
+        <v>20211118</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -25913,20 +25517,16 @@
       <c r="J101" t="n">
         <v>26</v>
       </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K101" t="n">
+        <v>10</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>2022-10-13</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr">
-        <is>
-          <t>20221013</t>
-        </is>
+      <c r="M101" t="n">
+        <v>20221013</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -26167,20 +25767,16 @@
       <c r="J102" t="n">
         <v>7</v>
       </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K102" t="n">
+        <v>10</v>
       </c>
       <c r="L102" t="inlineStr">
         <is>
           <t>2022-10-16</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr">
-        <is>
-          <t>20221016</t>
-        </is>
+      <c r="M102" t="n">
+        <v>20221016</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -26421,20 +26017,16 @@
       <c r="J103" t="n">
         <v>8</v>
       </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K103" t="n">
+        <v>10</v>
       </c>
       <c r="L103" t="inlineStr">
         <is>
           <t>2022-10-17</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr">
-        <is>
-          <t>20221017</t>
-        </is>
+      <c r="M103" t="n">
+        <v>20221017</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -26677,20 +26269,16 @@
       <c r="J104" t="n">
         <v>9</v>
       </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K104" t="n">
+        <v>10</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
           <t>2022-10-19</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr">
-        <is>
-          <t>20221019</t>
-        </is>
+      <c r="M104" t="n">
+        <v>20221019</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -26933,20 +26521,16 @@
       <c r="J105" t="n">
         <v>10</v>
       </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K105" t="n">
+        <v>10</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
           <t>2022-10-20</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr">
-        <is>
-          <t>20221020</t>
-        </is>
+      <c r="M105" t="n">
+        <v>20221020</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -27187,20 +26771,16 @@
       <c r="J106" t="n">
         <v>11</v>
       </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K106" t="n">
+        <v>10</v>
       </c>
       <c r="L106" t="inlineStr">
         <is>
           <t>2022-10-22</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr">
-        <is>
-          <t>20221022</t>
-        </is>
+      <c r="M106" t="n">
+        <v>20221022</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -27441,20 +27021,16 @@
       <c r="J107" t="n">
         <v>12</v>
       </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K107" t="n">
+        <v>10</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
           <t>2022-10-24</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr">
-        <is>
-          <t>20221024</t>
-        </is>
+      <c r="M107" t="n">
+        <v>20221024</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -27695,20 +27271,16 @@
       <c r="J108" t="n">
         <v>13</v>
       </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K108" t="n">
+        <v>10</v>
       </c>
       <c r="L108" t="inlineStr">
         <is>
           <t>2022-10-25</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr">
-        <is>
-          <t>20221025</t>
-        </is>
+      <c r="M108" t="n">
+        <v>20221025</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -27951,20 +27523,16 @@
       <c r="J109" t="n">
         <v>14</v>
       </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K109" t="n">
+        <v>10</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
           <t>2022-10-27</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr">
-        <is>
-          <t>20221027</t>
-        </is>
+      <c r="M109" t="n">
+        <v>20221027</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -28205,20 +27773,16 @@
       <c r="J110" t="n">
         <v>15</v>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K110" t="n">
+        <v>10</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>2022-10-28</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr">
-        <is>
-          <t>20221028</t>
-        </is>
+      <c r="M110" t="n">
+        <v>20221028</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -28459,20 +28023,16 @@
       <c r="J111" t="n">
         <v>19</v>
       </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K111" t="n">
+        <v>11</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
           <t>2022-11-01</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr">
-        <is>
-          <t>20221101</t>
-        </is>
+      <c r="M111" t="n">
+        <v>20221101</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -28719,20 +28279,16 @@
       <c r="J112" t="n">
         <v>20</v>
       </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K112" t="n">
+        <v>11</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
           <t>2022-11-02</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr">
-        <is>
-          <t>20221102</t>
-        </is>
+      <c r="M112" t="n">
+        <v>20221102</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -28973,20 +28529,16 @@
       <c r="J113" t="n">
         <v>21</v>
       </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K113" t="n">
+        <v>11</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
           <t>2022-11-04</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr">
-        <is>
-          <t>20221104</t>
-        </is>
+      <c r="M113" t="n">
+        <v>20221104</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -29229,20 +28781,16 @@
       <c r="J114" t="n">
         <v>22</v>
       </c>
-      <c r="K114" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K114" t="n">
+        <v>11</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>2022-11-05</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr">
-        <is>
-          <t>20221105</t>
-        </is>
+      <c r="M114" t="n">
+        <v>20221105</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -29483,20 +29031,16 @@
       <c r="J115" t="n">
         <v>23</v>
       </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K115" t="n">
+        <v>11</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
           <t>2022-11-07</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr">
-        <is>
-          <t>20221107</t>
-        </is>
+      <c r="M115" t="n">
+        <v>20221107</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -29739,20 +29283,16 @@
       <c r="J116" t="n">
         <v>24</v>
       </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K116" t="n">
+        <v>11</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
           <t>2022-11-08</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr">
-        <is>
-          <t>20221108</t>
-        </is>
+      <c r="M116" t="n">
+        <v>20221108</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -29993,20 +29533,16 @@
       <c r="J117" t="n">
         <v>26</v>
       </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K117" t="n">
+        <v>10</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
           <t>2023-10-19</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr">
-        <is>
-          <t>20231019</t>
-        </is>
+      <c r="M117" t="n">
+        <v>20231019</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
@@ -30247,20 +29783,16 @@
       <c r="J118" t="n">
         <v>7</v>
       </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K118" t="n">
+        <v>10</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
           <t>2023-10-22</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr">
-        <is>
-          <t>20231022</t>
-        </is>
+      <c r="M118" t="n">
+        <v>20231022</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
@@ -30503,20 +30035,16 @@
       <c r="J119" t="n">
         <v>8</v>
       </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K119" t="n">
+        <v>10</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
           <t>2023-10-23</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr">
-        <is>
-          <t>20231023</t>
-        </is>
+      <c r="M119" t="n">
+        <v>20231023</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -30759,20 +30287,16 @@
       <c r="J120" t="n">
         <v>9</v>
       </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K120" t="n">
+        <v>10</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
           <t>2023-10-25</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr">
-        <is>
-          <t>20231025</t>
-        </is>
+      <c r="M120" t="n">
+        <v>20231025</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -31013,20 +30537,16 @@
       <c r="J121" t="n">
         <v>12</v>
       </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K121" t="n">
+        <v>10</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
           <t>2023-10-30</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr">
-        <is>
-          <t>20231030</t>
-        </is>
+      <c r="M121" t="n">
+        <v>20231030</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -31269,20 +30789,16 @@
       <c r="J122" t="n">
         <v>13</v>
       </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K122" t="n">
+        <v>10</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
           <t>2023-10-31</t>
         </is>
       </c>
-      <c r="M122" t="inlineStr">
-        <is>
-          <t>20231031</t>
-        </is>
+      <c r="M122" t="n">
+        <v>20231031</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -31525,20 +31041,16 @@
       <c r="J123" t="n">
         <v>14</v>
       </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K123" t="n">
+        <v>11</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
           <t>2023-11-02</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr">
-        <is>
-          <t>20231102</t>
-        </is>
+      <c r="M123" t="n">
+        <v>20231102</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
@@ -31781,20 +31293,16 @@
       <c r="J124" t="n">
         <v>15</v>
       </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K124" t="n">
+        <v>11</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
           <t>2023-11-03</t>
         </is>
       </c>
-      <c r="M124" t="inlineStr">
-        <is>
-          <t>20231103</t>
-        </is>
+      <c r="M124" t="n">
+        <v>20231103</v>
       </c>
       <c r="N124" t="inlineStr">
         <is>
@@ -32037,20 +31545,16 @@
       <c r="J125" t="n">
         <v>16</v>
       </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K125" t="n">
+        <v>11</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
           <t>2023-11-05</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr">
-        <is>
-          <t>20231105</t>
-        </is>
+      <c r="M125" t="n">
+        <v>20231105</v>
       </c>
       <c r="N125" t="inlineStr">
         <is>
@@ -32291,20 +31795,16 @@
       <c r="J126" t="n">
         <v>19</v>
       </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K126" t="n">
+        <v>11</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
           <t>2023-11-07</t>
         </is>
       </c>
-      <c r="M126" t="inlineStr">
-        <is>
-          <t>20231107</t>
-        </is>
+      <c r="M126" t="n">
+        <v>20231107</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
@@ -32547,20 +32047,16 @@
       <c r="J127" t="n">
         <v>20</v>
       </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K127" t="n">
+        <v>11</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
           <t>2023-11-08</t>
         </is>
       </c>
-      <c r="M127" t="inlineStr">
-        <is>
-          <t>20231108</t>
-        </is>
+      <c r="M127" t="n">
+        <v>20231108</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -32801,20 +32297,16 @@
       <c r="J128" t="n">
         <v>21</v>
       </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K128" t="n">
+        <v>11</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
           <t>2023-11-10</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr">
-        <is>
-          <t>20231110</t>
-        </is>
+      <c r="M128" t="n">
+        <v>20231110</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -33057,20 +32549,16 @@
       <c r="J129" t="n">
         <v>22</v>
       </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K129" t="n">
+        <v>11</v>
       </c>
       <c r="L129" t="inlineStr">
         <is>
           <t>2023-11-11</t>
         </is>
       </c>
-      <c r="M129" t="inlineStr">
-        <is>
-          <t>20231111</t>
-        </is>
+      <c r="M129" t="n">
+        <v>20231111</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -33313,20 +32801,16 @@
       <c r="J130" t="n">
         <v>23</v>
       </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="K130" t="n">
+        <v>11</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
           <t>2023-11-13</t>
         </is>
       </c>
-      <c r="M130" t="inlineStr">
-        <is>
-          <t>20231113</t>
-        </is>
+      <c r="M130" t="n">
+        <v>20231113</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -33567,20 +33051,16 @@
       <c r="J131" t="n">
         <v>26</v>
       </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K131" t="n">
+        <v>10</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
           <t>2024-10-02</t>
         </is>
       </c>
-      <c r="M131" t="inlineStr">
-        <is>
-          <t>20241002</t>
-        </is>
+      <c r="M131" t="n">
+        <v>20241002</v>
       </c>
       <c r="N131" t="inlineStr">
         <is>
@@ -33823,20 +33303,16 @@
       <c r="J132" t="n">
         <v>27</v>
       </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K132" t="n">
+        <v>10</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
           <t>2024-10-03</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr">
-        <is>
-          <t>20241003</t>
-        </is>
+      <c r="M132" t="n">
+        <v>20241003</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -34079,20 +33555,16 @@
       <c r="J133" t="n">
         <v>7</v>
       </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K133" t="n">
+        <v>10</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
           <t>2024-10-05</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>20241005</t>
-        </is>
+      <c r="M133" t="n">
+        <v>20241005</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
@@ -34335,20 +33807,16 @@
       <c r="J134" t="n">
         <v>8</v>
       </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K134" t="n">
+        <v>10</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
           <t>2024-10-06</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
-        <is>
-          <t>20241006</t>
-        </is>
+      <c r="M134" t="n">
+        <v>20241006</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -34589,20 +34057,16 @@
       <c r="J135" t="n">
         <v>9</v>
       </c>
-      <c r="K135" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K135" t="n">
+        <v>10</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
           <t>2024-10-08</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr">
-        <is>
-          <t>20241008</t>
-        </is>
+      <c r="M135" t="n">
+        <v>20241008</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
@@ -34845,20 +34309,16 @@
       <c r="J136" t="n">
         <v>10</v>
       </c>
-      <c r="K136" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K136" t="n">
+        <v>10</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
           <t>2024-10-09</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr">
-        <is>
-          <t>20241009</t>
-        </is>
+      <c r="M136" t="n">
+        <v>20241009</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -35109,20 +34569,16 @@
       <c r="J137" t="n">
         <v>11</v>
       </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K137" t="n">
+        <v>10</v>
       </c>
       <c r="L137" t="inlineStr">
         <is>
           <t>2024-10-11</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr">
-        <is>
-          <t>20241011</t>
-        </is>
+      <c r="M137" t="n">
+        <v>20241011</v>
       </c>
       <c r="N137" t="inlineStr">
         <is>
@@ -35363,20 +34819,16 @@
       <c r="J138" t="n">
         <v>12</v>
       </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K138" t="n">
+        <v>10</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
           <t>2024-10-13</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr">
-        <is>
-          <t>20241013</t>
-        </is>
+      <c r="M138" t="n">
+        <v>20241013</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
@@ -35617,20 +35069,16 @@
       <c r="J139" t="n">
         <v>13</v>
       </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K139" t="n">
+        <v>10</v>
       </c>
       <c r="L139" t="inlineStr">
         <is>
           <t>2024-10-15</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr">
-        <is>
-          <t>20241015</t>
-        </is>
+      <c r="M139" t="n">
+        <v>20241015</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -35871,20 +35319,16 @@
       <c r="J140" t="n">
         <v>14</v>
       </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K140" t="n">
+        <v>10</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
           <t>2024-10-17</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr">
-        <is>
-          <t>20241017</t>
-        </is>
+      <c r="M140" t="n">
+        <v>20241017</v>
       </c>
       <c r="N140" t="inlineStr">
         <is>
@@ -36125,20 +35569,16 @@
       <c r="J141" t="n">
         <v>15</v>
       </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K141" t="n">
+        <v>10</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>
           <t>2024-10-19</t>
         </is>
       </c>
-      <c r="M141" t="inlineStr">
-        <is>
-          <t>20241019</t>
-        </is>
+      <c r="M141" t="n">
+        <v>20241019</v>
       </c>
       <c r="N141" t="inlineStr">
         <is>
@@ -36381,20 +35821,16 @@
       <c r="J142" t="n">
         <v>19</v>
       </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K142" t="n">
+        <v>10</v>
       </c>
       <c r="L142" t="inlineStr">
         <is>
           <t>2024-10-21</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr">
-        <is>
-          <t>20241021</t>
-        </is>
+      <c r="M142" t="n">
+        <v>20241021</v>
       </c>
       <c r="N142" t="inlineStr">
         <is>
@@ -36635,20 +36071,16 @@
       <c r="J143" t="n">
         <v>20</v>
       </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K143" t="n">
+        <v>10</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
           <t>2024-10-23</t>
         </is>
       </c>
-      <c r="M143" t="inlineStr">
-        <is>
-          <t>20241023</t>
-        </is>
+      <c r="M143" t="n">
+        <v>20241023</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -36889,20 +36321,16 @@
       <c r="J144" t="n">
         <v>21</v>
       </c>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K144" t="n">
+        <v>10</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
           <t>2024-10-25</t>
         </is>
       </c>
-      <c r="M144" t="inlineStr">
-        <is>
-          <t>20241025</t>
-        </is>
+      <c r="M144" t="n">
+        <v>20241025</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -37143,20 +36571,16 @@
       <c r="J145" t="n">
         <v>22</v>
       </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K145" t="n">
+        <v>10</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
           <t>2024-10-26</t>
         </is>
       </c>
-      <c r="M145" t="inlineStr">
-        <is>
-          <t>20241026</t>
-        </is>
+      <c r="M145" t="n">
+        <v>20241026</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -37399,20 +36823,16 @@
       <c r="J146" t="n">
         <v>23</v>
       </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K146" t="n">
+        <v>10</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
           <t>2024-10-28</t>
         </is>
       </c>
-      <c r="M146" t="inlineStr">
-        <is>
-          <t>20241028</t>
-        </is>
+      <c r="M146" t="n">
+        <v>20241028</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
@@ -37653,20 +37073,16 @@
       <c r="J147" t="n">
         <v>26</v>
       </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K147" t="n">
+        <v>10</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
           <t>2025-10-06</t>
         </is>
       </c>
-      <c r="M147" t="inlineStr">
-        <is>
-          <t>20251006</t>
-        </is>
+      <c r="M147" t="n">
+        <v>20251006</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
@@ -37909,20 +37325,16 @@
       <c r="J148" t="n">
         <v>27</v>
       </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K148" t="n">
+        <v>10</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
           <t>2025-10-07</t>
         </is>
       </c>
-      <c r="M148" t="inlineStr">
-        <is>
-          <t>20251007</t>
-        </is>
+      <c r="M148" t="n">
+        <v>20251007</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -38163,20 +37575,16 @@
       <c r="J149" t="n">
         <v>7</v>
       </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K149" t="n">
+        <v>10</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
           <t>2025-10-09</t>
         </is>
       </c>
-      <c r="M149" t="inlineStr">
-        <is>
-          <t>20251009</t>
-        </is>
+      <c r="M149" t="n">
+        <v>20251009</v>
       </c>
       <c r="N149" t="inlineStr">
         <is>
@@ -38419,20 +37827,16 @@
       <c r="J150" t="n">
         <v>8</v>
       </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K150" t="n">
+        <v>10</v>
       </c>
       <c r="L150" t="inlineStr">
         <is>
           <t>2025-10-11</t>
         </is>
       </c>
-      <c r="M150" t="inlineStr">
-        <is>
-          <t>20251011</t>
-        </is>
+      <c r="M150" t="n">
+        <v>20251011</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -38675,20 +38079,16 @@
       <c r="J151" t="n">
         <v>9</v>
       </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K151" t="n">
+        <v>10</v>
       </c>
       <c r="L151" t="inlineStr">
         <is>
           <t>2025-10-13</t>
         </is>
       </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t>20251013</t>
-        </is>
+      <c r="M151" t="n">
+        <v>20251013</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -38929,20 +38329,16 @@
       <c r="J152" t="n">
         <v>10</v>
       </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K152" t="n">
+        <v>10</v>
       </c>
       <c r="L152" t="inlineStr">
         <is>
           <t>2025-10-14</t>
         </is>
       </c>
-      <c r="M152" t="inlineStr">
-        <is>
-          <t>20251014</t>
-        </is>
+      <c r="M152" t="n">
+        <v>20251014</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -39183,20 +38579,16 @@
       <c r="J153" t="n">
         <v>12</v>
       </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K153" t="n">
+        <v>10</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
           <t>2025-10-18</t>
         </is>
       </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>20251018</t>
-        </is>
+      <c r="M153" t="n">
+        <v>20251018</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -39437,20 +38829,16 @@
       <c r="J154" t="n">
         <v>13</v>
       </c>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K154" t="n">
+        <v>10</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
           <t>2025-10-19</t>
         </is>
       </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t>20251019</t>
-        </is>
+      <c r="M154" t="n">
+        <v>20251019</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -39693,20 +39081,16 @@
       <c r="J155" t="n">
         <v>14</v>
       </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K155" t="n">
+        <v>10</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
           <t>2025-10-21</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr">
-        <is>
-          <t>20251021</t>
-        </is>
+      <c r="M155" t="n">
+        <v>20251021</v>
       </c>
       <c r="N155" t="inlineStr">
         <is>
@@ -39949,20 +39333,16 @@
       <c r="J156" t="n">
         <v>15</v>
       </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K156" t="n">
+        <v>10</v>
       </c>
       <c r="L156" t="inlineStr">
         <is>
           <t>2025-10-22</t>
         </is>
       </c>
-      <c r="M156" t="inlineStr">
-        <is>
-          <t>20251022</t>
-        </is>
+      <c r="M156" t="n">
+        <v>20251022</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -40203,20 +39583,16 @@
       <c r="J157" t="n">
         <v>16</v>
       </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K157" t="n">
+        <v>10</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
           <t>2025-10-24</t>
         </is>
       </c>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>20251024</t>
-        </is>
+      <c r="M157" t="n">
+        <v>20251024</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -40457,20 +39833,16 @@
       <c r="J158" t="n">
         <v>19</v>
       </c>
-      <c r="K158" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K158" t="n">
+        <v>10</v>
       </c>
       <c r="L158" t="inlineStr">
         <is>
           <t>2025-10-26</t>
         </is>
       </c>
-      <c r="M158" t="inlineStr">
-        <is>
-          <t>20251026</t>
-        </is>
+      <c r="M158" t="n">
+        <v>20251026</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -40711,20 +40083,16 @@
       <c r="J159" t="n">
         <v>20</v>
       </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K159" t="n">
+        <v>10</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
           <t>2025-10-27</t>
         </is>
       </c>
-      <c r="M159" t="inlineStr">
-        <is>
-          <t>20251027</t>
-        </is>
+      <c r="M159" t="n">
+        <v>20251027</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -40965,20 +40333,16 @@
       <c r="J160" t="n">
         <v>21</v>
       </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K160" t="n">
+        <v>10</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
           <t>2025-10-29</t>
         </is>
       </c>
-      <c r="M160" t="inlineStr">
-        <is>
-          <t>20251029</t>
-        </is>
+      <c r="M160" t="n">
+        <v>20251029</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -41219,20 +40583,16 @@
       <c r="J161" t="n">
         <v>22</v>
       </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K161" t="n">
+        <v>10</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
           <t>2025-10-30</t>
         </is>
       </c>
-      <c r="M161" t="inlineStr">
-        <is>
-          <t>20251030</t>
-        </is>
+      <c r="M161" t="n">
+        <v>20251030</v>
       </c>
       <c r="N161" t="inlineStr">
         <is>
@@ -41475,20 +40835,16 @@
       <c r="J162" t="n">
         <v>23</v>
       </c>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="K162" t="n">
+        <v>10</v>
       </c>
       <c r="L162" t="inlineStr">
         <is>
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="M162" t="inlineStr">
-        <is>
-          <t>20251031</t>
-        </is>
+      <c r="M162" t="n">
+        <v>20251031</v>
       </c>
       <c r="N162" t="inlineStr">
         <is>
@@ -41685,6 +41041,314 @@
       </c>
       <c r="BY162" t="inlineStr"/>
       <c r="BZ162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>20261014OBLG0</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>postseason</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>4</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>와일드카드 결정전</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>WC1</t>
+        </is>
+      </c>
+      <c r="H163" t="n">
+        <v>1</v>
+      </c>
+      <c r="I163" t="n">
+        <v>1</v>
+      </c>
+      <c r="J163" t="n">
+        <v>26</v>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>20261014</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>수</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr"/>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr"/>
+      <c r="T163" t="inlineStr"/>
+      <c r="U163" t="inlineStr"/>
+      <c r="V163" t="inlineStr"/>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>두산</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr"/>
+      <c r="Y163" t="inlineStr"/>
+      <c r="Z163" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="AA163" t="inlineStr"/>
+      <c r="AB163" t="inlineStr"/>
+      <c r="AC163" t="inlineStr"/>
+      <c r="AD163" t="inlineStr"/>
+      <c r="AE163" t="inlineStr"/>
+      <c r="AF163" t="inlineStr"/>
+      <c r="AG163" t="inlineStr"/>
+      <c r="AH163" t="inlineStr"/>
+      <c r="AI163" t="inlineStr"/>
+      <c r="AJ163" t="inlineStr"/>
+      <c r="AK163" t="inlineStr"/>
+      <c r="AL163" t="inlineStr"/>
+      <c r="AM163" t="inlineStr"/>
+      <c r="AN163" t="inlineStr"/>
+      <c r="AO163" t="inlineStr"/>
+      <c r="AP163" t="inlineStr"/>
+      <c r="AQ163" t="inlineStr"/>
+      <c r="AR163" t="inlineStr"/>
+      <c r="AS163" t="inlineStr"/>
+      <c r="AT163" t="inlineStr"/>
+      <c r="AU163" t="inlineStr"/>
+      <c r="AV163" t="inlineStr"/>
+      <c r="AW163" t="inlineStr"/>
+      <c r="AX163" t="inlineStr"/>
+      <c r="AY163" t="inlineStr"/>
+      <c r="AZ163" t="inlineStr"/>
+      <c r="BA163" t="inlineStr"/>
+      <c r="BB163" t="inlineStr"/>
+      <c r="BC163" t="inlineStr"/>
+      <c r="BD163" t="inlineStr"/>
+      <c r="BE163" t="inlineStr"/>
+      <c r="BF163" t="inlineStr"/>
+      <c r="BG163" t="inlineStr"/>
+      <c r="BH163" t="inlineStr"/>
+      <c r="BI163" t="inlineStr"/>
+      <c r="BJ163" t="inlineStr"/>
+      <c r="BK163" t="inlineStr"/>
+      <c r="BL163" t="inlineStr"/>
+      <c r="BM163" t="inlineStr"/>
+      <c r="BN163" t="inlineStr"/>
+      <c r="BO163" t="inlineStr"/>
+      <c r="BP163" t="inlineStr"/>
+      <c r="BQ163" t="inlineStr"/>
+      <c r="BR163" t="inlineStr"/>
+      <c r="BS163" t="inlineStr"/>
+      <c r="BT163" t="inlineStr"/>
+      <c r="BU163" t="inlineStr">
+        <is>
+          <t>preview</t>
+        </is>
+      </c>
+      <c r="BV163" t="inlineStr"/>
+      <c r="BW163" t="inlineStr">
+        <is>
+          <t>잠실</t>
+        </is>
+      </c>
+      <c r="BX163" t="inlineStr"/>
+      <c r="BY163" t="inlineStr"/>
+      <c r="BZ163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>20261015OBLG0</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>postseason</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>4</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>와일드카드 결정전</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>WC2</t>
+        </is>
+      </c>
+      <c r="H164" t="n">
+        <v>2</v>
+      </c>
+      <c r="I164" t="n">
+        <v>1</v>
+      </c>
+      <c r="J164" t="n">
+        <v>27</v>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>20261015</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>목</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr"/>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr"/>
+      <c r="T164" t="inlineStr"/>
+      <c r="U164" t="inlineStr"/>
+      <c r="V164" t="inlineStr"/>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>두산</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr"/>
+      <c r="Y164" t="inlineStr"/>
+      <c r="Z164" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="AA164" t="inlineStr"/>
+      <c r="AB164" t="inlineStr"/>
+      <c r="AC164" t="inlineStr"/>
+      <c r="AD164" t="inlineStr"/>
+      <c r="AE164" t="inlineStr"/>
+      <c r="AF164" t="inlineStr"/>
+      <c r="AG164" t="inlineStr"/>
+      <c r="AH164" t="inlineStr"/>
+      <c r="AI164" t="inlineStr"/>
+      <c r="AJ164" t="inlineStr"/>
+      <c r="AK164" t="inlineStr"/>
+      <c r="AL164" t="inlineStr"/>
+      <c r="AM164" t="inlineStr"/>
+      <c r="AN164" t="inlineStr"/>
+      <c r="AO164" t="inlineStr"/>
+      <c r="AP164" t="inlineStr"/>
+      <c r="AQ164" t="inlineStr"/>
+      <c r="AR164" t="inlineStr"/>
+      <c r="AS164" t="inlineStr"/>
+      <c r="AT164" t="inlineStr"/>
+      <c r="AU164" t="inlineStr"/>
+      <c r="AV164" t="inlineStr"/>
+      <c r="AW164" t="inlineStr"/>
+      <c r="AX164" t="inlineStr"/>
+      <c r="AY164" t="inlineStr"/>
+      <c r="AZ164" t="inlineStr"/>
+      <c r="BA164" t="inlineStr"/>
+      <c r="BB164" t="inlineStr"/>
+      <c r="BC164" t="inlineStr"/>
+      <c r="BD164" t="inlineStr"/>
+      <c r="BE164" t="inlineStr"/>
+      <c r="BF164" t="inlineStr"/>
+      <c r="BG164" t="inlineStr"/>
+      <c r="BH164" t="inlineStr"/>
+      <c r="BI164" t="inlineStr"/>
+      <c r="BJ164" t="inlineStr"/>
+      <c r="BK164" t="inlineStr"/>
+      <c r="BL164" t="inlineStr"/>
+      <c r="BM164" t="inlineStr"/>
+      <c r="BN164" t="inlineStr"/>
+      <c r="BO164" t="inlineStr"/>
+      <c r="BP164" t="inlineStr"/>
+      <c r="BQ164" t="inlineStr"/>
+      <c r="BR164" t="inlineStr"/>
+      <c r="BS164" t="inlineStr"/>
+      <c r="BT164" t="inlineStr"/>
+      <c r="BU164" t="inlineStr">
+        <is>
+          <t>preview</t>
+        </is>
+      </c>
+      <c r="BV164" t="inlineStr"/>
+      <c r="BW164" t="inlineStr">
+        <is>
+          <t>잠실</t>
+        </is>
+      </c>
+      <c r="BX164" t="inlineStr"/>
+      <c r="BY164" t="inlineStr"/>
+      <c r="BZ164" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>